<commit_message>
Remove unused legacy files from app source
</commit_message>
<xml_diff>
--- a/tools/Alle standen derde divisie.xlsx
+++ b/tools/Alle standen derde divisie.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ngijs\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ngijs\derde_divisie\tools\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D0F78B68-6A81-4DAF-AA31-B36DB856586C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A0C7031B-F69F-46E0-A7CA-D716578610B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{E185487E-D128-410B-AABE-8B50484F0E01}"/>
   </bookViews>
@@ -607,9 +607,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
@@ -643,6 +640,9 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -983,7 +983,7 @@
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="17.33203125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="8.88671875" style="24"/>
+    <col min="11" max="11" width="8.88671875" style="23"/>
     <col min="13" max="13" width="18.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -993,92 +993,92 @@
       </c>
     </row>
     <row r="2" spans="1:22" x14ac:dyDescent="0.3">
-      <c r="A2" s="6" t="s">
+      <c r="A2" s="27" t="s">
         <v>19</v>
       </c>
-      <c r="B2" s="6"/>
-      <c r="C2" s="6"/>
-      <c r="D2" s="6"/>
-      <c r="E2" s="6"/>
-      <c r="F2" s="6"/>
-      <c r="G2" s="6"/>
-      <c r="H2" s="6"/>
-      <c r="I2" s="6"/>
-      <c r="J2" s="6"/>
-      <c r="K2" s="26"/>
-      <c r="M2" s="6" t="s">
+      <c r="B2" s="27"/>
+      <c r="C2" s="27"/>
+      <c r="D2" s="27"/>
+      <c r="E2" s="27"/>
+      <c r="F2" s="27"/>
+      <c r="G2" s="27"/>
+      <c r="H2" s="27"/>
+      <c r="I2" s="27"/>
+      <c r="J2" s="27"/>
+      <c r="K2" s="25"/>
+      <c r="M2" s="27" t="s">
         <v>20</v>
       </c>
-      <c r="N2" s="6"/>
-      <c r="O2" s="6"/>
-      <c r="P2" s="6"/>
-      <c r="Q2" s="6"/>
-      <c r="R2" s="6"/>
-      <c r="S2" s="6"/>
-      <c r="T2" s="6"/>
-      <c r="U2" s="6"/>
-      <c r="V2" s="6"/>
+      <c r="N2" s="27"/>
+      <c r="O2" s="27"/>
+      <c r="P2" s="27"/>
+      <c r="Q2" s="27"/>
+      <c r="R2" s="27"/>
+      <c r="S2" s="27"/>
+      <c r="T2" s="27"/>
+      <c r="U2" s="27"/>
+      <c r="V2" s="27"/>
     </row>
     <row r="3" spans="1:22" x14ac:dyDescent="0.3">
-      <c r="A3" s="27" t="s">
+      <c r="A3" s="26" t="s">
         <v>139</v>
       </c>
-      <c r="B3" s="12" t="s">
+      <c r="B3" s="11" t="s">
         <v>130</v>
       </c>
-      <c r="C3" s="12" t="s">
+      <c r="C3" s="11" t="s">
         <v>131</v>
       </c>
-      <c r="D3" s="12" t="s">
+      <c r="D3" s="11" t="s">
         <v>132</v>
       </c>
-      <c r="E3" s="12" t="s">
+      <c r="E3" s="11" t="s">
         <v>133</v>
       </c>
-      <c r="F3" s="12" t="s">
+      <c r="F3" s="11" t="s">
         <v>134</v>
       </c>
-      <c r="G3" s="12" t="s">
+      <c r="G3" s="11" t="s">
         <v>135</v>
       </c>
-      <c r="H3" s="12" t="s">
+      <c r="H3" s="11" t="s">
         <v>136</v>
       </c>
-      <c r="I3" s="12" t="s">
+      <c r="I3" s="11" t="s">
         <v>137</v>
       </c>
-      <c r="J3" s="12" t="s">
+      <c r="J3" s="11" t="s">
         <v>138</v>
       </c>
-      <c r="K3" s="25"/>
-      <c r="L3" s="25" t="s">
+      <c r="K3" s="24"/>
+      <c r="L3" s="24" t="s">
         <v>139</v>
       </c>
-      <c r="M3" s="12" t="s">
+      <c r="M3" s="11" t="s">
         <v>130</v>
       </c>
-      <c r="N3" s="12" t="s">
+      <c r="N3" s="11" t="s">
         <v>131</v>
       </c>
-      <c r="O3" s="12" t="s">
+      <c r="O3" s="11" t="s">
         <v>132</v>
       </c>
-      <c r="P3" s="12" t="s">
+      <c r="P3" s="11" t="s">
         <v>133</v>
       </c>
-      <c r="Q3" s="12" t="s">
+      <c r="Q3" s="11" t="s">
         <v>134</v>
       </c>
-      <c r="R3" s="12" t="s">
+      <c r="R3" s="11" t="s">
         <v>135</v>
       </c>
-      <c r="S3" s="12" t="s">
+      <c r="S3" s="11" t="s">
         <v>136</v>
       </c>
-      <c r="T3" s="12" t="s">
+      <c r="T3" s="11" t="s">
         <v>137</v>
       </c>
-      <c r="U3" s="12" t="s">
+      <c r="U3" s="11" t="s">
         <v>138</v>
       </c>
       <c r="V3" s="5"/>
@@ -2337,32 +2337,32 @@
       </c>
     </row>
     <row r="25" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="B25" s="7" t="s">
+      <c r="B25" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="C25" s="7">
-        <v>34</v>
-      </c>
-      <c r="D25" s="7">
+      <c r="C25" s="6">
+        <v>34</v>
+      </c>
+      <c r="D25" s="6">
         <v>20</v>
       </c>
-      <c r="E25" s="7">
+      <c r="E25" s="6">
         <v>5</v>
       </c>
-      <c r="F25" s="7">
+      <c r="F25" s="6">
         <v>9</v>
       </c>
-      <c r="G25" s="7">
+      <c r="G25" s="6">
         <f t="shared" ref="G25:G40" si="7">D25*3+E25</f>
         <v>65</v>
       </c>
-      <c r="H25" s="7">
+      <c r="H25" s="6">
         <v>68</v>
       </c>
-      <c r="I25" s="7">
+      <c r="I25" s="6">
         <v>44</v>
       </c>
-      <c r="J25" s="7">
+      <c r="J25" s="6">
         <f t="shared" ref="J25:J41" si="8">H25-I25</f>
         <v>24</v>
       </c>
@@ -2467,32 +2467,32 @@
       </c>
     </row>
     <row r="27" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="B27" s="7" t="s">
+      <c r="B27" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="C27" s="7">
-        <v>34</v>
-      </c>
-      <c r="D27" s="7">
+      <c r="C27" s="6">
+        <v>34</v>
+      </c>
+      <c r="D27" s="6">
         <v>18</v>
       </c>
-      <c r="E27" s="7">
+      <c r="E27" s="6">
         <v>7</v>
       </c>
-      <c r="F27" s="7">
+      <c r="F27" s="6">
         <v>9</v>
       </c>
-      <c r="G27" s="7">
+      <c r="G27" s="6">
         <f t="shared" si="7"/>
         <v>61</v>
       </c>
-      <c r="H27" s="7">
+      <c r="H27" s="6">
         <v>73</v>
       </c>
-      <c r="I27" s="7">
+      <c r="I27" s="6">
         <v>54</v>
       </c>
-      <c r="J27" s="7">
+      <c r="J27" s="6">
         <f t="shared" si="8"/>
         <v>19</v>
       </c>
@@ -2662,32 +2662,32 @@
       </c>
     </row>
     <row r="30" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="B30" s="7" t="s">
+      <c r="B30" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="C30" s="7">
-        <v>34</v>
-      </c>
-      <c r="D30" s="7">
+      <c r="C30" s="6">
+        <v>34</v>
+      </c>
+      <c r="D30" s="6">
         <v>18</v>
       </c>
-      <c r="E30" s="7">
+      <c r="E30" s="6">
         <v>2</v>
       </c>
-      <c r="F30" s="7">
+      <c r="F30" s="6">
         <v>14</v>
       </c>
-      <c r="G30" s="7">
+      <c r="G30" s="6">
         <f t="shared" si="7"/>
         <v>56</v>
       </c>
-      <c r="H30" s="7">
+      <c r="H30" s="6">
         <v>60</v>
       </c>
-      <c r="I30" s="7">
+      <c r="I30" s="6">
         <v>48</v>
       </c>
-      <c r="J30" s="7">
+      <c r="J30" s="6">
         <f t="shared" si="8"/>
         <v>12</v>
       </c>
@@ -3516,32 +3516,32 @@
       </c>
     </row>
     <row r="44" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="B44" s="7" t="s">
+      <c r="B44" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="C44" s="7">
-        <v>34</v>
-      </c>
-      <c r="D44" s="7">
+      <c r="C44" s="6">
+        <v>34</v>
+      </c>
+      <c r="D44" s="6">
         <v>22</v>
       </c>
-      <c r="E44" s="7">
+      <c r="E44" s="6">
         <v>6</v>
       </c>
-      <c r="F44" s="7">
+      <c r="F44" s="6">
         <v>6</v>
       </c>
-      <c r="G44" s="7">
+      <c r="G44" s="6">
         <f t="shared" ref="G44:G59" si="12">D44*3+E44</f>
         <v>72</v>
       </c>
-      <c r="H44" s="7">
+      <c r="H44" s="6">
         <v>84</v>
       </c>
-      <c r="I44" s="7">
+      <c r="I44" s="6">
         <v>40</v>
       </c>
-      <c r="J44" s="7">
+      <c r="J44" s="6">
         <f t="shared" ref="J44:J60" si="13">H44-I44</f>
         <v>44</v>
       </c>
@@ -3646,32 +3646,32 @@
       </c>
     </row>
     <row r="46" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="B46" s="7" t="s">
+      <c r="B46" s="6" t="s">
         <v>55</v>
       </c>
-      <c r="C46" s="7">
-        <v>34</v>
-      </c>
-      <c r="D46" s="7">
+      <c r="C46" s="6">
+        <v>34</v>
+      </c>
+      <c r="D46" s="6">
         <v>19</v>
       </c>
-      <c r="E46" s="7">
+      <c r="E46" s="6">
         <v>7</v>
       </c>
-      <c r="F46" s="7">
+      <c r="F46" s="6">
         <v>8</v>
       </c>
-      <c r="G46" s="7">
+      <c r="G46" s="6">
         <f t="shared" si="12"/>
         <v>64</v>
       </c>
-      <c r="H46" s="7">
+      <c r="H46" s="6">
         <v>82</v>
       </c>
-      <c r="I46" s="7">
+      <c r="I46" s="6">
         <v>55</v>
       </c>
-      <c r="J46" s="7">
+      <c r="J46" s="6">
         <f t="shared" si="13"/>
         <v>27</v>
       </c>
@@ -3841,32 +3841,32 @@
       </c>
     </row>
     <row r="49" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="B49" s="7" t="s">
+      <c r="B49" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="C49" s="7">
-        <v>34</v>
-      </c>
-      <c r="D49" s="7">
+      <c r="C49" s="6">
+        <v>34</v>
+      </c>
+      <c r="D49" s="6">
         <v>16</v>
       </c>
-      <c r="E49" s="7">
+      <c r="E49" s="6">
         <v>7</v>
       </c>
-      <c r="F49" s="7">
+      <c r="F49" s="6">
         <v>11</v>
       </c>
-      <c r="G49" s="7">
+      <c r="G49" s="6">
         <f t="shared" si="12"/>
         <v>55</v>
       </c>
-      <c r="H49" s="7">
+      <c r="H49" s="6">
         <v>74</v>
       </c>
-      <c r="I49" s="7">
+      <c r="I49" s="6">
         <v>54</v>
       </c>
-      <c r="J49" s="7">
+      <c r="J49" s="6">
         <f t="shared" si="13"/>
         <v>20</v>
       </c>
@@ -4695,32 +4695,32 @@
       </c>
     </row>
     <row r="63" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="B63" s="8" t="s">
+      <c r="B63" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="C63" s="8">
+      <c r="C63" s="7">
         <v>22</v>
       </c>
-      <c r="D63" s="8">
+      <c r="D63" s="7">
         <v>15</v>
       </c>
-      <c r="E63" s="8">
+      <c r="E63" s="7">
         <v>2</v>
       </c>
-      <c r="F63" s="8">
+      <c r="F63" s="7">
         <v>5</v>
       </c>
-      <c r="G63" s="8">
+      <c r="G63" s="7">
         <f t="shared" ref="G63:G78" si="17">D63*3+E63</f>
         <v>47</v>
       </c>
-      <c r="H63" s="8">
+      <c r="H63" s="7">
         <v>63</v>
       </c>
-      <c r="I63" s="8">
+      <c r="I63" s="7">
         <v>30</v>
       </c>
-      <c r="J63" s="8">
+      <c r="J63" s="7">
         <f t="shared" ref="J63:J78" si="18">H63-I63</f>
         <v>33</v>
       </c>
@@ -4760,32 +4760,32 @@
       </c>
     </row>
     <row r="64" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="B64" s="8" t="s">
+      <c r="B64" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="C64" s="8">
+      <c r="C64" s="7">
         <v>22</v>
       </c>
-      <c r="D64" s="8">
+      <c r="D64" s="7">
         <v>13</v>
       </c>
-      <c r="E64" s="8">
+      <c r="E64" s="7">
         <v>3</v>
       </c>
-      <c r="F64" s="8">
+      <c r="F64" s="7">
         <v>6</v>
       </c>
-      <c r="G64" s="8">
+      <c r="G64" s="7">
         <f t="shared" si="17"/>
         <v>42</v>
       </c>
-      <c r="H64" s="8">
+      <c r="H64" s="7">
         <v>43</v>
       </c>
-      <c r="I64" s="8">
-        <v>34</v>
-      </c>
-      <c r="J64" s="8">
+      <c r="I64" s="7">
+        <v>34</v>
+      </c>
+      <c r="J64" s="7">
         <f t="shared" si="18"/>
         <v>9</v>
       </c>
@@ -4825,32 +4825,32 @@
       </c>
     </row>
     <row r="65" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="B65" s="8" t="s">
+      <c r="B65" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="C65" s="8">
+      <c r="C65" s="7">
         <v>23</v>
       </c>
-      <c r="D65" s="8">
+      <c r="D65" s="7">
         <v>13</v>
       </c>
-      <c r="E65" s="8">
+      <c r="E65" s="7">
         <v>3</v>
       </c>
-      <c r="F65" s="8">
+      <c r="F65" s="7">
         <v>7</v>
       </c>
-      <c r="G65" s="8">
+      <c r="G65" s="7">
         <f t="shared" si="17"/>
         <v>42</v>
       </c>
-      <c r="H65" s="8">
+      <c r="H65" s="7">
         <v>39</v>
       </c>
-      <c r="I65" s="8">
+      <c r="I65" s="7">
         <v>30</v>
       </c>
-      <c r="J65" s="8">
+      <c r="J65" s="7">
         <f t="shared" si="18"/>
         <v>9</v>
       </c>
@@ -5809,32 +5809,32 @@
       </c>
     </row>
     <row r="81" spans="2:21" x14ac:dyDescent="0.3">
-      <c r="B81" s="8" t="s">
+      <c r="B81" s="7" t="s">
         <v>2</v>
       </c>
-      <c r="C81" s="8">
+      <c r="C81" s="7">
         <v>5</v>
       </c>
-      <c r="D81" s="8">
+      <c r="D81" s="7">
         <v>3</v>
       </c>
-      <c r="E81" s="8">
+      <c r="E81" s="7">
         <v>1</v>
       </c>
-      <c r="F81" s="8">
+      <c r="F81" s="7">
         <v>1</v>
       </c>
-      <c r="G81" s="8">
+      <c r="G81" s="7">
         <f t="shared" ref="G81:G97" si="23">D81*3+E81</f>
         <v>10</v>
       </c>
-      <c r="H81" s="8">
+      <c r="H81" s="7">
         <v>11</v>
       </c>
-      <c r="I81" s="8">
+      <c r="I81" s="7">
         <v>7</v>
       </c>
-      <c r="J81" s="8">
+      <c r="J81" s="7">
         <f t="shared" ref="J81:J97" si="24">H81-I81</f>
         <v>4</v>
       </c>
@@ -5874,32 +5874,32 @@
       </c>
     </row>
     <row r="82" spans="2:21" x14ac:dyDescent="0.3">
-      <c r="B82" s="8" t="s">
+      <c r="B82" s="7" t="s">
         <v>65</v>
       </c>
-      <c r="C82" s="8">
+      <c r="C82" s="7">
         <v>5</v>
       </c>
-      <c r="D82" s="8">
+      <c r="D82" s="7">
         <v>3</v>
       </c>
-      <c r="E82" s="8">
+      <c r="E82" s="7">
         <v>1</v>
       </c>
-      <c r="F82" s="8">
+      <c r="F82" s="7">
         <v>1</v>
       </c>
-      <c r="G82" s="8">
+      <c r="G82" s="7">
         <f t="shared" si="23"/>
         <v>10</v>
       </c>
-      <c r="H82" s="8">
+      <c r="H82" s="7">
         <v>9</v>
       </c>
-      <c r="I82" s="8">
+      <c r="I82" s="7">
         <v>5</v>
       </c>
-      <c r="J82" s="8">
+      <c r="J82" s="7">
         <f t="shared" si="24"/>
         <v>4</v>
       </c>
@@ -5939,32 +5939,32 @@
       </c>
     </row>
     <row r="83" spans="2:21" x14ac:dyDescent="0.3">
-      <c r="B83" s="8" t="s">
+      <c r="B83" s="7" t="s">
         <v>67</v>
       </c>
-      <c r="C83" s="8">
+      <c r="C83" s="7">
         <v>5</v>
       </c>
-      <c r="D83" s="8">
+      <c r="D83" s="7">
         <v>3</v>
       </c>
-      <c r="E83" s="8">
+      <c r="E83" s="7">
         <v>1</v>
       </c>
-      <c r="F83" s="8">
+      <c r="F83" s="7">
         <v>1</v>
       </c>
-      <c r="G83" s="8">
+      <c r="G83" s="7">
         <f t="shared" si="23"/>
         <v>10</v>
       </c>
-      <c r="H83" s="8">
+      <c r="H83" s="7">
         <v>8</v>
       </c>
-      <c r="I83" s="8">
+      <c r="I83" s="7">
         <v>5</v>
       </c>
-      <c r="J83" s="8">
+      <c r="J83" s="7">
         <f t="shared" si="24"/>
         <v>3</v>
       </c>
@@ -6926,7 +6926,7 @@
       <c r="B99" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="C99" s="9">
+      <c r="C99" s="8">
         <v>34</v>
       </c>
       <c r="D99" s="1">
@@ -6938,7 +6938,7 @@
       <c r="F99" s="1">
         <v>6</v>
       </c>
-      <c r="G99" s="9">
+      <c r="G99" s="8">
         <f>D99*3+E99</f>
         <v>70</v>
       </c>
@@ -6948,11 +6948,11 @@
       <c r="I99" s="1">
         <v>38</v>
       </c>
-      <c r="J99" s="9">
+      <c r="J99" s="8">
         <f>H99-I99</f>
         <v>32</v>
       </c>
-      <c r="K99" s="25"/>
+      <c r="K99" s="24"/>
       <c r="L99" t="str">
         <f t="shared" si="21"/>
         <v>2021/22</v>
@@ -6960,65 +6960,65 @@
       <c r="M99" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="N99" s="15">
-        <v>34</v>
-      </c>
-      <c r="O99" s="15">
+      <c r="N99" s="14">
+        <v>34</v>
+      </c>
+      <c r="O99" s="14">
         <v>18</v>
       </c>
-      <c r="P99" s="15">
+      <c r="P99" s="14">
         <v>7</v>
       </c>
-      <c r="Q99" s="15">
+      <c r="Q99" s="14">
         <f>N99-O99-P99</f>
         <v>9</v>
       </c>
-      <c r="R99" s="15">
+      <c r="R99" s="14">
         <f t="shared" ref="R99:R116" si="27">O99*3+P99*1</f>
         <v>61</v>
       </c>
-      <c r="S99" s="15">
+      <c r="S99" s="14">
         <v>66</v>
       </c>
-      <c r="T99" s="15">
+      <c r="T99" s="14">
         <v>47</v>
       </c>
-      <c r="U99" s="15">
+      <c r="U99" s="14">
         <f>S99-T99</f>
         <v>19</v>
       </c>
     </row>
     <row r="100" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="B100" s="10" t="s">
+      <c r="B100" s="9" t="s">
         <v>65</v>
       </c>
-      <c r="C100" s="11">
-        <v>34</v>
-      </c>
-      <c r="D100" s="10">
+      <c r="C100" s="10">
+        <v>34</v>
+      </c>
+      <c r="D100" s="9">
         <v>19</v>
       </c>
-      <c r="E100" s="10">
+      <c r="E100" s="9">
         <v>7</v>
       </c>
-      <c r="F100" s="10">
+      <c r="F100" s="9">
         <v>8</v>
       </c>
-      <c r="G100" s="11">
+      <c r="G100" s="10">
         <f t="shared" ref="G100:G116" si="28">D100*3+E100</f>
         <v>64</v>
       </c>
-      <c r="H100" s="10">
+      <c r="H100" s="9">
         <v>65</v>
       </c>
-      <c r="I100" s="10">
+      <c r="I100" s="9">
         <v>38</v>
       </c>
-      <c r="J100" s="11">
+      <c r="J100" s="10">
         <f t="shared" ref="J100:J116" si="29">H100-I100</f>
         <v>27</v>
       </c>
-      <c r="K100" s="25"/>
+      <c r="K100" s="24"/>
       <c r="L100" t="str">
         <f t="shared" si="21"/>
         <v/>
@@ -7026,65 +7026,65 @@
       <c r="M100" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="N100" s="16">
-        <v>34</v>
-      </c>
-      <c r="O100" s="16">
+      <c r="N100" s="15">
+        <v>34</v>
+      </c>
+      <c r="O100" s="15">
         <v>18</v>
       </c>
-      <c r="P100" s="16">
+      <c r="P100" s="15">
         <v>5</v>
       </c>
-      <c r="Q100" s="16">
+      <c r="Q100" s="15">
         <f t="shared" ref="Q100:Q116" si="30">N100-O100-P100</f>
         <v>11</v>
       </c>
-      <c r="R100" s="16">
+      <c r="R100" s="15">
         <f t="shared" si="27"/>
         <v>59</v>
       </c>
-      <c r="S100" s="16">
+      <c r="S100" s="15">
         <v>74</v>
       </c>
-      <c r="T100" s="16">
+      <c r="T100" s="15">
         <v>46</v>
       </c>
-      <c r="U100" s="16">
+      <c r="U100" s="15">
         <f t="shared" ref="U100:U116" si="31">S100-T100</f>
         <v>28</v>
       </c>
     </row>
     <row r="101" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="B101" s="10" t="s">
+      <c r="B101" s="9" t="s">
         <v>77</v>
       </c>
-      <c r="C101" s="11">
-        <v>34</v>
-      </c>
-      <c r="D101" s="10">
+      <c r="C101" s="10">
+        <v>34</v>
+      </c>
+      <c r="D101" s="9">
         <v>17</v>
       </c>
-      <c r="E101" s="10">
+      <c r="E101" s="9">
         <v>7</v>
       </c>
-      <c r="F101" s="10">
+      <c r="F101" s="9">
         <v>10</v>
       </c>
-      <c r="G101" s="11">
+      <c r="G101" s="10">
         <f t="shared" si="28"/>
         <v>58</v>
       </c>
-      <c r="H101" s="10">
+      <c r="H101" s="9">
         <v>63</v>
       </c>
-      <c r="I101" s="10">
+      <c r="I101" s="9">
         <v>40</v>
       </c>
-      <c r="J101" s="11">
+      <c r="J101" s="10">
         <f t="shared" si="29"/>
         <v>23</v>
       </c>
-      <c r="K101" s="25"/>
+      <c r="K101" s="24"/>
       <c r="L101" t="str">
         <f t="shared" si="21"/>
         <v/>
@@ -7092,65 +7092,65 @@
       <c r="M101" t="s">
         <v>49</v>
       </c>
-      <c r="N101" s="17">
-        <v>34</v>
-      </c>
-      <c r="O101" s="17">
+      <c r="N101" s="16">
+        <v>34</v>
+      </c>
+      <c r="O101" s="16">
         <v>17</v>
       </c>
-      <c r="P101" s="17">
+      <c r="P101" s="16">
         <v>7</v>
       </c>
-      <c r="Q101" s="17">
+      <c r="Q101" s="16">
         <f t="shared" si="30"/>
         <v>10</v>
       </c>
-      <c r="R101" s="17">
+      <c r="R101" s="16">
         <f t="shared" si="27"/>
         <v>58</v>
       </c>
-      <c r="S101" s="17">
+      <c r="S101" s="16">
         <v>64</v>
       </c>
-      <c r="T101" s="17">
+      <c r="T101" s="16">
         <v>46</v>
       </c>
-      <c r="U101" s="17">
+      <c r="U101" s="16">
         <f t="shared" si="31"/>
         <v>18</v>
       </c>
     </row>
     <row r="102" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="B102" s="10" t="s">
+      <c r="B102" s="9" t="s">
         <v>7</v>
       </c>
-      <c r="C102" s="11">
-        <v>34</v>
-      </c>
-      <c r="D102" s="10">
+      <c r="C102" s="10">
+        <v>34</v>
+      </c>
+      <c r="D102" s="9">
         <v>18</v>
       </c>
-      <c r="E102" s="10">
+      <c r="E102" s="9">
         <v>4</v>
       </c>
-      <c r="F102" s="10">
+      <c r="F102" s="9">
         <v>12</v>
       </c>
-      <c r="G102" s="11">
+      <c r="G102" s="10">
         <f t="shared" si="28"/>
         <v>58</v>
       </c>
-      <c r="H102" s="10">
+      <c r="H102" s="9">
         <v>61</v>
       </c>
-      <c r="I102" s="10">
+      <c r="I102" s="9">
         <v>41</v>
       </c>
-      <c r="J102" s="11">
+      <c r="J102" s="10">
         <f t="shared" si="29"/>
         <v>20</v>
       </c>
-      <c r="K102" s="25"/>
+      <c r="K102" s="24"/>
       <c r="L102" t="str">
         <f t="shared" si="21"/>
         <v/>
@@ -7158,30 +7158,30 @@
       <c r="M102" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="N102" s="16">
-        <v>34</v>
-      </c>
-      <c r="O102" s="16">
+      <c r="N102" s="15">
+        <v>34</v>
+      </c>
+      <c r="O102" s="15">
         <v>15</v>
       </c>
-      <c r="P102" s="16">
+      <c r="P102" s="15">
         <v>12</v>
       </c>
-      <c r="Q102" s="16">
+      <c r="Q102" s="15">
         <f t="shared" si="30"/>
         <v>7</v>
       </c>
-      <c r="R102" s="16">
+      <c r="R102" s="15">
         <f t="shared" si="27"/>
         <v>57</v>
       </c>
-      <c r="S102" s="16">
+      <c r="S102" s="15">
         <v>75</v>
       </c>
-      <c r="T102" s="16">
+      <c r="T102" s="15">
         <v>57</v>
       </c>
-      <c r="U102" s="16">
+      <c r="U102" s="15">
         <f t="shared" si="31"/>
         <v>18</v>
       </c>
@@ -7190,7 +7190,7 @@
       <c r="B103" t="s">
         <v>55</v>
       </c>
-      <c r="C103" s="12">
+      <c r="C103" s="11">
         <v>34</v>
       </c>
       <c r="D103">
@@ -7202,7 +7202,7 @@
       <c r="F103">
         <v>11</v>
       </c>
-      <c r="G103" s="12">
+      <c r="G103" s="11">
         <f t="shared" si="28"/>
         <v>55</v>
       </c>
@@ -7212,11 +7212,11 @@
       <c r="I103">
         <v>49</v>
       </c>
-      <c r="J103" s="12">
+      <c r="J103" s="11">
         <f t="shared" si="29"/>
         <v>4</v>
       </c>
-      <c r="K103" s="25"/>
+      <c r="K103" s="24"/>
       <c r="L103" t="str">
         <f t="shared" si="21"/>
         <v/>
@@ -7224,30 +7224,30 @@
       <c r="M103" t="s">
         <v>62</v>
       </c>
-      <c r="N103" s="17">
-        <v>34</v>
-      </c>
-      <c r="O103" s="17">
+      <c r="N103" s="16">
+        <v>34</v>
+      </c>
+      <c r="O103" s="16">
         <v>16</v>
       </c>
-      <c r="P103" s="17">
+      <c r="P103" s="16">
         <v>8</v>
       </c>
-      <c r="Q103" s="17">
+      <c r="Q103" s="16">
         <f t="shared" si="30"/>
         <v>10</v>
       </c>
-      <c r="R103" s="17">
+      <c r="R103" s="16">
         <f t="shared" si="27"/>
         <v>56</v>
       </c>
-      <c r="S103" s="17">
+      <c r="S103" s="16">
         <v>62</v>
       </c>
-      <c r="T103" s="17">
+      <c r="T103" s="16">
         <v>46</v>
       </c>
-      <c r="U103" s="17">
+      <c r="U103" s="16">
         <f t="shared" si="31"/>
         <v>16</v>
       </c>
@@ -7256,7 +7256,7 @@
       <c r="B104" t="s">
         <v>44</v>
       </c>
-      <c r="C104" s="12">
+      <c r="C104" s="11">
         <v>34</v>
       </c>
       <c r="D104">
@@ -7268,7 +7268,7 @@
       <c r="F104">
         <v>11</v>
       </c>
-      <c r="G104" s="12">
+      <c r="G104" s="11">
         <f t="shared" si="28"/>
         <v>51</v>
       </c>
@@ -7278,11 +7278,11 @@
       <c r="I104">
         <v>42</v>
       </c>
-      <c r="J104" s="12">
+      <c r="J104" s="11">
         <f t="shared" si="29"/>
         <v>8</v>
       </c>
-      <c r="K104" s="25"/>
+      <c r="K104" s="24"/>
       <c r="L104" t="str">
         <f t="shared" si="21"/>
         <v/>
@@ -7290,30 +7290,30 @@
       <c r="M104" t="s">
         <v>73</v>
       </c>
-      <c r="N104" s="17">
-        <v>34</v>
-      </c>
-      <c r="O104" s="17">
+      <c r="N104" s="16">
+        <v>34</v>
+      </c>
+      <c r="O104" s="16">
         <v>14</v>
       </c>
-      <c r="P104" s="17">
+      <c r="P104" s="16">
         <v>9</v>
       </c>
-      <c r="Q104" s="17">
+      <c r="Q104" s="16">
         <f t="shared" si="30"/>
         <v>11</v>
       </c>
-      <c r="R104" s="17">
+      <c r="R104" s="16">
         <f>O104*3+P104*1</f>
         <v>51</v>
       </c>
-      <c r="S104" s="17">
+      <c r="S104" s="16">
         <v>48</v>
       </c>
-      <c r="T104" s="17">
+      <c r="T104" s="16">
         <v>50</v>
       </c>
-      <c r="U104" s="17">
+      <c r="U104" s="16">
         <f t="shared" si="31"/>
         <v>-2</v>
       </c>
@@ -7322,7 +7322,7 @@
       <c r="B105" t="s">
         <v>67</v>
       </c>
-      <c r="C105" s="12">
+      <c r="C105" s="11">
         <v>34</v>
       </c>
       <c r="D105">
@@ -7334,7 +7334,7 @@
       <c r="F105">
         <v>11</v>
       </c>
-      <c r="G105" s="12">
+      <c r="G105" s="11">
         <f t="shared" si="28"/>
         <v>51</v>
       </c>
@@ -7344,11 +7344,11 @@
       <c r="I105">
         <v>47</v>
       </c>
-      <c r="J105" s="12">
+      <c r="J105" s="11">
         <f t="shared" si="29"/>
         <v>6</v>
       </c>
-      <c r="K105" s="25"/>
+      <c r="K105" s="24"/>
       <c r="L105" t="str">
         <f t="shared" si="21"/>
         <v/>
@@ -7356,30 +7356,30 @@
       <c r="M105" t="s">
         <v>23</v>
       </c>
-      <c r="N105" s="17">
-        <v>34</v>
-      </c>
-      <c r="O105" s="17">
+      <c r="N105" s="16">
+        <v>34</v>
+      </c>
+      <c r="O105" s="16">
         <v>13</v>
       </c>
-      <c r="P105" s="17">
+      <c r="P105" s="16">
         <v>11</v>
       </c>
-      <c r="Q105" s="17">
+      <c r="Q105" s="16">
         <f t="shared" si="30"/>
         <v>10</v>
       </c>
-      <c r="R105" s="17">
+      <c r="R105" s="16">
         <f t="shared" si="27"/>
         <v>50</v>
       </c>
-      <c r="S105" s="17">
+      <c r="S105" s="16">
         <v>56</v>
       </c>
-      <c r="T105" s="17">
+      <c r="T105" s="16">
         <v>47</v>
       </c>
-      <c r="U105" s="17">
+      <c r="U105" s="16">
         <f t="shared" si="31"/>
         <v>9</v>
       </c>
@@ -7388,7 +7388,7 @@
       <c r="B106" t="s">
         <v>66</v>
       </c>
-      <c r="C106" s="12">
+      <c r="C106" s="11">
         <v>34</v>
       </c>
       <c r="D106">
@@ -7400,7 +7400,7 @@
       <c r="F106">
         <v>10</v>
       </c>
-      <c r="G106" s="12">
+      <c r="G106" s="11">
         <f t="shared" si="28"/>
         <v>50</v>
       </c>
@@ -7410,11 +7410,11 @@
       <c r="I106">
         <v>57</v>
       </c>
-      <c r="J106" s="12">
+      <c r="J106" s="11">
         <f t="shared" si="29"/>
         <v>15</v>
       </c>
-      <c r="K106" s="25"/>
+      <c r="K106" s="24"/>
       <c r="L106" t="str">
         <f t="shared" si="21"/>
         <v/>
@@ -7422,30 +7422,30 @@
       <c r="M106" t="s">
         <v>47</v>
       </c>
-      <c r="N106" s="17">
-        <v>34</v>
-      </c>
-      <c r="O106" s="17">
+      <c r="N106" s="16">
+        <v>34</v>
+      </c>
+      <c r="O106" s="16">
         <v>15</v>
       </c>
-      <c r="P106" s="17">
+      <c r="P106" s="16">
         <v>5</v>
       </c>
-      <c r="Q106" s="17">
+      <c r="Q106" s="16">
         <f t="shared" si="30"/>
         <v>14</v>
       </c>
-      <c r="R106" s="17">
+      <c r="R106" s="16">
         <f t="shared" si="27"/>
         <v>50</v>
       </c>
-      <c r="S106" s="17">
+      <c r="S106" s="16">
         <v>60</v>
       </c>
-      <c r="T106" s="17">
+      <c r="T106" s="16">
         <v>58</v>
       </c>
-      <c r="U106" s="17">
+      <c r="U106" s="16">
         <f t="shared" si="31"/>
         <v>2</v>
       </c>
@@ -7454,7 +7454,7 @@
       <c r="B107" t="s">
         <v>16</v>
       </c>
-      <c r="C107" s="12">
+      <c r="C107" s="11">
         <v>34</v>
       </c>
       <c r="D107">
@@ -7466,7 +7466,7 @@
       <c r="F107">
         <v>13</v>
       </c>
-      <c r="G107" s="12">
+      <c r="G107" s="11">
         <f t="shared" si="28"/>
         <v>45</v>
       </c>
@@ -7476,11 +7476,11 @@
       <c r="I107">
         <v>48</v>
       </c>
-      <c r="J107" s="12">
+      <c r="J107" s="11">
         <f t="shared" si="29"/>
         <v>1</v>
       </c>
-      <c r="K107" s="25"/>
+      <c r="K107" s="24"/>
       <c r="L107" t="str">
         <f t="shared" si="21"/>
         <v/>
@@ -7488,30 +7488,30 @@
       <c r="M107" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="N107" s="16">
-        <v>34</v>
-      </c>
-      <c r="O107" s="16">
+      <c r="N107" s="15">
+        <v>34</v>
+      </c>
+      <c r="O107" s="15">
         <v>15</v>
       </c>
-      <c r="P107" s="16">
+      <c r="P107" s="15">
         <v>4</v>
       </c>
-      <c r="Q107" s="16">
+      <c r="Q107" s="15">
         <f t="shared" si="30"/>
         <v>15</v>
       </c>
-      <c r="R107" s="16">
+      <c r="R107" s="15">
         <f t="shared" si="27"/>
         <v>49</v>
       </c>
-      <c r="S107" s="16">
+      <c r="S107" s="15">
         <v>63</v>
       </c>
-      <c r="T107" s="16">
+      <c r="T107" s="15">
         <v>52</v>
       </c>
-      <c r="U107" s="16">
+      <c r="U107" s="15">
         <f t="shared" si="31"/>
         <v>11</v>
       </c>
@@ -7520,7 +7520,7 @@
       <c r="B108" t="s">
         <v>78</v>
       </c>
-      <c r="C108" s="12">
+      <c r="C108" s="11">
         <v>34</v>
       </c>
       <c r="D108">
@@ -7532,7 +7532,7 @@
       <c r="F108">
         <v>15</v>
       </c>
-      <c r="G108" s="12">
+      <c r="G108" s="11">
         <f t="shared" si="28"/>
         <v>45</v>
       </c>
@@ -7542,11 +7542,11 @@
       <c r="I108">
         <v>56</v>
       </c>
-      <c r="J108" s="12">
+      <c r="J108" s="11">
         <f t="shared" si="29"/>
         <v>-2</v>
       </c>
-      <c r="K108" s="25"/>
+      <c r="K108" s="24"/>
       <c r="L108" t="str">
         <f t="shared" si="21"/>
         <v/>
@@ -7554,30 +7554,30 @@
       <c r="M108" t="s">
         <v>74</v>
       </c>
-      <c r="N108" s="17">
-        <v>34</v>
-      </c>
-      <c r="O108" s="17">
+      <c r="N108" s="16">
+        <v>34</v>
+      </c>
+      <c r="O108" s="16">
         <v>14</v>
       </c>
-      <c r="P108" s="17">
+      <c r="P108" s="16">
         <v>5</v>
       </c>
-      <c r="Q108" s="17">
+      <c r="Q108" s="16">
         <f t="shared" si="30"/>
         <v>15</v>
       </c>
-      <c r="R108" s="17">
+      <c r="R108" s="16">
         <f t="shared" si="27"/>
         <v>47</v>
       </c>
-      <c r="S108" s="17">
+      <c r="S108" s="16">
         <v>47</v>
       </c>
-      <c r="T108" s="17">
+      <c r="T108" s="16">
         <v>44</v>
       </c>
-      <c r="U108" s="17">
+      <c r="U108" s="16">
         <f t="shared" si="31"/>
         <v>3</v>
       </c>
@@ -7586,7 +7586,7 @@
       <c r="B109" t="s">
         <v>69</v>
       </c>
-      <c r="C109" s="12">
+      <c r="C109" s="11">
         <v>34</v>
       </c>
       <c r="D109">
@@ -7598,7 +7598,7 @@
       <c r="F109">
         <v>16</v>
       </c>
-      <c r="G109" s="12">
+      <c r="G109" s="11">
         <f t="shared" si="28"/>
         <v>44</v>
       </c>
@@ -7608,11 +7608,11 @@
       <c r="I109">
         <v>67</v>
       </c>
-      <c r="J109" s="12">
+      <c r="J109" s="11">
         <f t="shared" si="29"/>
         <v>-18</v>
       </c>
-      <c r="K109" s="25"/>
+      <c r="K109" s="24"/>
       <c r="L109" t="str">
         <f t="shared" si="21"/>
         <v/>
@@ -7620,30 +7620,30 @@
       <c r="M109" t="s">
         <v>63</v>
       </c>
-      <c r="N109" s="17">
-        <v>34</v>
-      </c>
-      <c r="O109" s="17">
+      <c r="N109" s="16">
+        <v>34</v>
+      </c>
+      <c r="O109" s="16">
         <v>13</v>
       </c>
-      <c r="P109" s="17">
+      <c r="P109" s="16">
         <v>6</v>
       </c>
-      <c r="Q109" s="17">
+      <c r="Q109" s="16">
         <f t="shared" si="30"/>
         <v>15</v>
       </c>
-      <c r="R109" s="17">
+      <c r="R109" s="16">
         <f t="shared" si="27"/>
         <v>45</v>
       </c>
-      <c r="S109" s="17">
+      <c r="S109" s="16">
         <v>55</v>
       </c>
-      <c r="T109" s="17">
+      <c r="T109" s="16">
         <v>56</v>
       </c>
-      <c r="U109" s="17">
+      <c r="U109" s="16">
         <f t="shared" si="31"/>
         <v>-1</v>
       </c>
@@ -7652,7 +7652,7 @@
       <c r="B110" t="s">
         <v>8</v>
       </c>
-      <c r="C110" s="12">
+      <c r="C110" s="11">
         <v>34</v>
       </c>
       <c r="D110">
@@ -7664,7 +7664,7 @@
       <c r="F110">
         <v>12</v>
       </c>
-      <c r="G110" s="12">
+      <c r="G110" s="11">
         <f t="shared" si="28"/>
         <v>42</v>
       </c>
@@ -7674,11 +7674,11 @@
       <c r="I110">
         <v>62</v>
       </c>
-      <c r="J110" s="12">
+      <c r="J110" s="11">
         <f t="shared" si="29"/>
         <v>1</v>
       </c>
-      <c r="K110" s="25"/>
+      <c r="K110" s="24"/>
       <c r="L110" t="str">
         <f t="shared" si="21"/>
         <v/>
@@ -7686,30 +7686,30 @@
       <c r="M110" t="s">
         <v>72</v>
       </c>
-      <c r="N110" s="17">
-        <v>34</v>
-      </c>
-      <c r="O110" s="17">
+      <c r="N110" s="16">
+        <v>34</v>
+      </c>
+      <c r="O110" s="16">
         <v>13</v>
       </c>
-      <c r="P110" s="17">
+      <c r="P110" s="16">
         <v>6</v>
       </c>
-      <c r="Q110" s="17">
+      <c r="Q110" s="16">
         <f t="shared" si="30"/>
         <v>15</v>
       </c>
-      <c r="R110" s="17">
+      <c r="R110" s="16">
         <f t="shared" si="27"/>
         <v>45</v>
       </c>
-      <c r="S110" s="17">
+      <c r="S110" s="16">
         <v>37</v>
       </c>
-      <c r="T110" s="17">
+      <c r="T110" s="16">
         <v>50</v>
       </c>
-      <c r="U110" s="17">
+      <c r="U110" s="16">
         <f t="shared" si="31"/>
         <v>-13</v>
       </c>
@@ -7718,7 +7718,7 @@
       <c r="B111" t="s">
         <v>40</v>
       </c>
-      <c r="C111" s="12">
+      <c r="C111" s="11">
         <v>34</v>
       </c>
       <c r="D111">
@@ -7730,7 +7730,7 @@
       <c r="F111">
         <v>16</v>
       </c>
-      <c r="G111" s="12">
+      <c r="G111" s="11">
         <f t="shared" si="28"/>
         <v>38</v>
       </c>
@@ -7740,11 +7740,11 @@
       <c r="I111">
         <v>57</v>
       </c>
-      <c r="J111" s="12">
+      <c r="J111" s="11">
         <f t="shared" si="29"/>
         <v>-14</v>
       </c>
-      <c r="K111" s="25"/>
+      <c r="K111" s="24"/>
       <c r="L111" t="str">
         <f t="shared" si="21"/>
         <v/>
@@ -7752,30 +7752,30 @@
       <c r="M111" t="s">
         <v>80</v>
       </c>
-      <c r="N111" s="17">
-        <v>34</v>
-      </c>
-      <c r="O111" s="17">
+      <c r="N111" s="16">
+        <v>34</v>
+      </c>
+      <c r="O111" s="16">
         <v>12</v>
       </c>
-      <c r="P111" s="17">
+      <c r="P111" s="16">
         <v>6</v>
       </c>
-      <c r="Q111" s="17">
+      <c r="Q111" s="16">
         <f t="shared" si="30"/>
         <v>16</v>
       </c>
-      <c r="R111" s="17">
+      <c r="R111" s="16">
         <f t="shared" si="27"/>
         <v>42</v>
       </c>
-      <c r="S111" s="17">
+      <c r="S111" s="16">
         <v>41</v>
       </c>
-      <c r="T111" s="17">
+      <c r="T111" s="16">
         <v>59</v>
       </c>
-      <c r="U111" s="17">
+      <c r="U111" s="16">
         <f t="shared" si="31"/>
         <v>-18</v>
       </c>
@@ -7784,7 +7784,7 @@
       <c r="B112" t="s">
         <v>68</v>
       </c>
-      <c r="C112" s="12">
+      <c r="C112" s="11">
         <v>34</v>
       </c>
       <c r="D112">
@@ -7796,7 +7796,7 @@
       <c r="F112">
         <v>16</v>
       </c>
-      <c r="G112" s="12">
+      <c r="G112" s="11">
         <f t="shared" si="28"/>
         <v>38</v>
       </c>
@@ -7806,11 +7806,11 @@
       <c r="I112">
         <v>66</v>
       </c>
-      <c r="J112" s="12">
+      <c r="J112" s="11">
         <f t="shared" si="29"/>
         <v>-16</v>
       </c>
-      <c r="K112" s="25"/>
+      <c r="K112" s="24"/>
       <c r="L112" t="str">
         <f t="shared" si="21"/>
         <v/>
@@ -7818,30 +7818,30 @@
       <c r="M112" t="s">
         <v>82</v>
       </c>
-      <c r="N112" s="17">
-        <v>34</v>
-      </c>
-      <c r="O112" s="17">
+      <c r="N112" s="16">
+        <v>34</v>
+      </c>
+      <c r="O112" s="16">
         <v>12</v>
       </c>
-      <c r="P112" s="17">
+      <c r="P112" s="16">
         <v>6</v>
       </c>
-      <c r="Q112" s="17">
+      <c r="Q112" s="16">
         <f t="shared" si="30"/>
         <v>16</v>
       </c>
-      <c r="R112" s="17">
+      <c r="R112" s="16">
         <f>O112*3+P112*1</f>
         <v>42</v>
       </c>
-      <c r="S112" s="17">
+      <c r="S112" s="16">
         <v>59</v>
       </c>
-      <c r="T112" s="17">
+      <c r="T112" s="16">
         <v>69</v>
       </c>
-      <c r="U112" s="17">
+      <c r="U112" s="16">
         <f t="shared" si="31"/>
         <v>-10</v>
       </c>
@@ -7850,7 +7850,7 @@
       <c r="B113" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="C113" s="13">
+      <c r="C113" s="12">
         <v>34</v>
       </c>
       <c r="D113" s="3">
@@ -7862,7 +7862,7 @@
       <c r="F113" s="3">
         <v>15</v>
       </c>
-      <c r="G113" s="13">
+      <c r="G113" s="12">
         <f t="shared" si="28"/>
         <v>37</v>
       </c>
@@ -7872,11 +7872,11 @@
       <c r="I113" s="3">
         <v>68</v>
       </c>
-      <c r="J113" s="13">
+      <c r="J113" s="12">
         <f t="shared" si="29"/>
         <v>-16</v>
       </c>
-      <c r="K113" s="25"/>
+      <c r="K113" s="24"/>
       <c r="L113" t="str">
         <f t="shared" si="21"/>
         <v/>
@@ -7884,30 +7884,30 @@
       <c r="M113" s="3" t="s">
         <v>76</v>
       </c>
-      <c r="N113" s="18">
-        <v>34</v>
-      </c>
-      <c r="O113" s="18">
+      <c r="N113" s="17">
+        <v>34</v>
+      </c>
+      <c r="O113" s="17">
         <v>11</v>
       </c>
-      <c r="P113" s="18">
+      <c r="P113" s="17">
         <v>6</v>
       </c>
-      <c r="Q113" s="18">
+      <c r="Q113" s="17">
         <f t="shared" si="30"/>
         <v>17</v>
       </c>
-      <c r="R113" s="18">
+      <c r="R113" s="17">
         <f t="shared" si="27"/>
         <v>39</v>
       </c>
-      <c r="S113" s="18">
+      <c r="S113" s="17">
         <v>42</v>
       </c>
-      <c r="T113" s="18">
+      <c r="T113" s="17">
         <v>64</v>
       </c>
-      <c r="U113" s="18">
+      <c r="U113" s="17">
         <f t="shared" si="31"/>
         <v>-22</v>
       </c>
@@ -7916,7 +7916,7 @@
       <c r="B114" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="C114" s="13">
+      <c r="C114" s="12">
         <v>34</v>
       </c>
       <c r="D114" s="3">
@@ -7928,7 +7928,7 @@
       <c r="F114" s="3">
         <v>17</v>
       </c>
-      <c r="G114" s="13">
+      <c r="G114" s="12">
         <f t="shared" si="28"/>
         <v>37</v>
       </c>
@@ -7938,11 +7938,11 @@
       <c r="I114" s="3">
         <v>82</v>
       </c>
-      <c r="J114" s="13">
+      <c r="J114" s="12">
         <f t="shared" si="29"/>
         <v>-21</v>
       </c>
-      <c r="K114" s="25"/>
+      <c r="K114" s="24"/>
       <c r="L114" t="str">
         <f t="shared" si="21"/>
         <v/>
@@ -7950,30 +7950,30 @@
       <c r="M114" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="N114" s="18">
-        <v>34</v>
-      </c>
-      <c r="O114" s="18">
+      <c r="N114" s="17">
+        <v>34</v>
+      </c>
+      <c r="O114" s="17">
         <v>9</v>
       </c>
-      <c r="P114" s="18">
+      <c r="P114" s="17">
         <v>10</v>
       </c>
-      <c r="Q114" s="18">
+      <c r="Q114" s="17">
         <f t="shared" si="30"/>
         <v>15</v>
       </c>
-      <c r="R114" s="18">
+      <c r="R114" s="17">
         <f t="shared" si="27"/>
         <v>37</v>
       </c>
-      <c r="S114" s="18">
+      <c r="S114" s="17">
         <v>36</v>
       </c>
-      <c r="T114" s="18">
+      <c r="T114" s="17">
         <v>59</v>
       </c>
-      <c r="U114" s="18">
+      <c r="U114" s="17">
         <f t="shared" si="31"/>
         <v>-23</v>
       </c>
@@ -7982,7 +7982,7 @@
       <c r="B115" s="4" t="s">
         <v>56</v>
       </c>
-      <c r="C115" s="14">
+      <c r="C115" s="13">
         <v>34</v>
       </c>
       <c r="D115" s="4">
@@ -7994,7 +7994,7 @@
       <c r="F115" s="4">
         <v>18</v>
       </c>
-      <c r="G115" s="14">
+      <c r="G115" s="13">
         <f t="shared" si="28"/>
         <v>36</v>
       </c>
@@ -8004,11 +8004,11 @@
       <c r="I115" s="4">
         <v>54</v>
       </c>
-      <c r="J115" s="14">
+      <c r="J115" s="13">
         <f t="shared" si="29"/>
         <v>-16</v>
       </c>
-      <c r="K115" s="25"/>
+      <c r="K115" s="24"/>
       <c r="L115" t="str">
         <f t="shared" si="21"/>
         <v/>
@@ -8016,30 +8016,30 @@
       <c r="M115" s="4" t="s">
         <v>81</v>
       </c>
-      <c r="N115" s="19">
-        <v>34</v>
-      </c>
-      <c r="O115" s="19">
+      <c r="N115" s="18">
+        <v>34</v>
+      </c>
+      <c r="O115" s="18">
         <v>10</v>
       </c>
-      <c r="P115" s="19">
+      <c r="P115" s="18">
         <v>5</v>
       </c>
-      <c r="Q115" s="19">
+      <c r="Q115" s="18">
         <f t="shared" si="30"/>
         <v>19</v>
       </c>
-      <c r="R115" s="19">
+      <c r="R115" s="18">
         <f t="shared" si="27"/>
         <v>35</v>
       </c>
-      <c r="S115" s="19">
+      <c r="S115" s="18">
         <v>38</v>
       </c>
-      <c r="T115" s="19">
+      <c r="T115" s="18">
         <v>55</v>
       </c>
-      <c r="U115" s="19">
+      <c r="U115" s="18">
         <f t="shared" si="31"/>
         <v>-17</v>
       </c>
@@ -8048,7 +8048,7 @@
       <c r="B116" s="4" t="s">
         <v>79</v>
       </c>
-      <c r="C116" s="14">
+      <c r="C116" s="13">
         <v>34</v>
       </c>
       <c r="D116" s="4">
@@ -8060,7 +8060,7 @@
       <c r="F116" s="4">
         <v>18</v>
       </c>
-      <c r="G116" s="14">
+      <c r="G116" s="13">
         <f t="shared" si="28"/>
         <v>28</v>
       </c>
@@ -8070,11 +8070,11 @@
       <c r="I116" s="4">
         <v>78</v>
       </c>
-      <c r="J116" s="14">
+      <c r="J116" s="13">
         <f t="shared" si="29"/>
         <v>-34</v>
       </c>
-      <c r="K116" s="25"/>
+      <c r="K116" s="24"/>
       <c r="L116" t="str">
         <f t="shared" si="21"/>
         <v/>
@@ -8082,30 +8082,30 @@
       <c r="M116" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="N116" s="19">
-        <v>34</v>
-      </c>
-      <c r="O116" s="19">
+      <c r="N116" s="18">
+        <v>34</v>
+      </c>
+      <c r="O116" s="18">
         <v>8</v>
       </c>
-      <c r="P116" s="19">
+      <c r="P116" s="18">
         <v>8</v>
       </c>
-      <c r="Q116" s="19">
+      <c r="Q116" s="18">
         <f t="shared" si="30"/>
         <v>18</v>
       </c>
-      <c r="R116" s="19">
+      <c r="R116" s="18">
         <f t="shared" si="27"/>
         <v>32</v>
       </c>
-      <c r="S116" s="19">
+      <c r="S116" s="18">
         <v>43</v>
       </c>
-      <c r="T116" s="19">
+      <c r="T116" s="18">
         <v>61</v>
       </c>
-      <c r="U116" s="19">
+      <c r="U116" s="18">
         <f t="shared" si="31"/>
         <v>-18</v>
       </c>
@@ -8123,7 +8123,7 @@
       <c r="B118" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="C118" s="9">
+      <c r="C118" s="8">
         <v>34</v>
       </c>
       <c r="D118" s="1">
@@ -8135,7 +8135,7 @@
       <c r="F118" s="1">
         <v>3</v>
       </c>
-      <c r="G118" s="9">
+      <c r="G118" s="8">
         <f>D118*3+E118</f>
         <v>75</v>
       </c>
@@ -8145,11 +8145,11 @@
       <c r="I118" s="1">
         <v>33</v>
       </c>
-      <c r="J118" s="9">
+      <c r="J118" s="8">
         <f t="shared" ref="J118:J135" si="32">H118-I118</f>
         <v>38</v>
       </c>
-      <c r="K118" s="25"/>
+      <c r="K118" s="24"/>
       <c r="L118" t="str">
         <f t="shared" si="21"/>
         <v>2022/23</v>
@@ -8189,7 +8189,7 @@
       <c r="B119" s="2" t="s">
         <v>84</v>
       </c>
-      <c r="C119" s="23">
+      <c r="C119" s="22">
         <v>34</v>
       </c>
       <c r="D119" s="2">
@@ -8201,7 +8201,7 @@
       <c r="F119" s="2">
         <v>7</v>
       </c>
-      <c r="G119" s="23">
+      <c r="G119" s="22">
         <f>D119*3+E119</f>
         <v>69</v>
       </c>
@@ -8211,11 +8211,11 @@
       <c r="I119" s="2">
         <v>40</v>
       </c>
-      <c r="J119" s="23">
+      <c r="J119" s="22">
         <f t="shared" si="32"/>
         <v>37</v>
       </c>
-      <c r="K119" s="25"/>
+      <c r="K119" s="24"/>
       <c r="L119" t="str">
         <f t="shared" si="21"/>
         <v/>
@@ -8255,7 +8255,7 @@
       <c r="B120" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="C120" s="23">
+      <c r="C120" s="22">
         <v>34</v>
       </c>
       <c r="D120" s="2">
@@ -8267,7 +8267,7 @@
       <c r="F120" s="2">
         <v>12</v>
       </c>
-      <c r="G120" s="23">
+      <c r="G120" s="22">
         <f>D120*3+E120</f>
         <v>58</v>
       </c>
@@ -8277,11 +8277,11 @@
       <c r="I120" s="2">
         <v>42</v>
       </c>
-      <c r="J120" s="23">
+      <c r="J120" s="22">
         <f t="shared" si="32"/>
         <v>17</v>
       </c>
-      <c r="K120" s="25"/>
+      <c r="K120" s="24"/>
       <c r="L120" t="str">
         <f t="shared" si="21"/>
         <v/>
@@ -8321,7 +8321,7 @@
       <c r="B121" t="s">
         <v>85</v>
       </c>
-      <c r="C121" s="12">
+      <c r="C121" s="11">
         <v>34</v>
       </c>
       <c r="D121">
@@ -8333,7 +8333,7 @@
       <c r="F121">
         <v>12</v>
       </c>
-      <c r="G121" s="12">
+      <c r="G121" s="11">
         <f>D121*3+E121</f>
         <v>56</v>
       </c>
@@ -8343,11 +8343,11 @@
       <c r="I121">
         <v>55</v>
       </c>
-      <c r="J121" s="12">
+      <c r="J121" s="11">
         <f t="shared" si="32"/>
         <v>9</v>
       </c>
-      <c r="K121" s="25"/>
+      <c r="K121" s="24"/>
       <c r="L121" t="str">
         <f t="shared" si="21"/>
         <v/>
@@ -8384,36 +8384,36 @@
       </c>
     </row>
     <row r="122" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="B122" s="24" t="s">
+      <c r="B122" s="23" t="s">
         <v>66</v>
       </c>
-      <c r="C122" s="25">
-        <v>34</v>
-      </c>
-      <c r="D122" s="24">
+      <c r="C122" s="24">
+        <v>34</v>
+      </c>
+      <c r="D122" s="23">
         <v>18</v>
       </c>
-      <c r="E122" s="24">
+      <c r="E122" s="23">
         <v>5</v>
       </c>
-      <c r="F122" s="24">
+      <c r="F122" s="23">
         <v>11</v>
       </c>
-      <c r="G122" s="25">
+      <c r="G122" s="24">
         <f>D122*3+E122-4</f>
         <v>55</v>
       </c>
-      <c r="H122" s="24">
+      <c r="H122" s="23">
         <v>71</v>
       </c>
-      <c r="I122" s="24">
+      <c r="I122" s="23">
         <v>54</v>
       </c>
-      <c r="J122" s="25">
+      <c r="J122" s="24">
         <f t="shared" si="32"/>
         <v>17</v>
       </c>
-      <c r="K122" s="25"/>
+      <c r="K122" s="24"/>
       <c r="L122" t="str">
         <f t="shared" si="21"/>
         <v/>
@@ -8453,7 +8453,7 @@
       <c r="B123" t="s">
         <v>86</v>
       </c>
-      <c r="C123" s="12">
+      <c r="C123" s="11">
         <v>34</v>
       </c>
       <c r="D123">
@@ -8465,7 +8465,7 @@
       <c r="F123">
         <v>11</v>
       </c>
-      <c r="G123" s="12">
+      <c r="G123" s="11">
         <f t="shared" ref="G123:G135" si="36">D123*3+E123</f>
         <v>53</v>
       </c>
@@ -8475,11 +8475,11 @@
       <c r="I123">
         <v>50</v>
       </c>
-      <c r="J123" s="12">
+      <c r="J123" s="11">
         <f t="shared" si="32"/>
         <v>2</v>
       </c>
-      <c r="K123" s="25"/>
+      <c r="K123" s="24"/>
       <c r="L123" t="str">
         <f t="shared" si="21"/>
         <v/>
@@ -8519,7 +8519,7 @@
       <c r="B124" t="s">
         <v>87</v>
       </c>
-      <c r="C124" s="12">
+      <c r="C124" s="11">
         <v>34</v>
       </c>
       <c r="D124">
@@ -8531,7 +8531,7 @@
       <c r="F124">
         <v>12</v>
       </c>
-      <c r="G124" s="12">
+      <c r="G124" s="11">
         <f t="shared" si="36"/>
         <v>52</v>
       </c>
@@ -8541,11 +8541,11 @@
       <c r="I124">
         <v>43</v>
       </c>
-      <c r="J124" s="12">
+      <c r="J124" s="11">
         <f t="shared" si="32"/>
         <v>11</v>
       </c>
-      <c r="K124" s="25"/>
+      <c r="K124" s="24"/>
       <c r="L124" t="str">
         <f t="shared" si="21"/>
         <v/>
@@ -8585,7 +8585,7 @@
       <c r="B125" t="s">
         <v>88</v>
       </c>
-      <c r="C125" s="12">
+      <c r="C125" s="11">
         <v>34</v>
       </c>
       <c r="D125">
@@ -8597,7 +8597,7 @@
       <c r="F125">
         <v>10</v>
       </c>
-      <c r="G125" s="12">
+      <c r="G125" s="11">
         <f t="shared" si="36"/>
         <v>50</v>
       </c>
@@ -8607,11 +8607,11 @@
       <c r="I125">
         <v>45</v>
       </c>
-      <c r="J125" s="12">
+      <c r="J125" s="11">
         <f t="shared" si="32"/>
         <v>0</v>
       </c>
-      <c r="K125" s="25"/>
+      <c r="K125" s="24"/>
       <c r="L125" t="str">
         <f t="shared" si="21"/>
         <v/>
@@ -8651,7 +8651,7 @@
       <c r="B126" t="s">
         <v>55</v>
       </c>
-      <c r="C126" s="12">
+      <c r="C126" s="11">
         <v>34</v>
       </c>
       <c r="D126">
@@ -8663,7 +8663,7 @@
       <c r="F126">
         <v>16</v>
       </c>
-      <c r="G126" s="12">
+      <c r="G126" s="11">
         <f t="shared" si="36"/>
         <v>50</v>
       </c>
@@ -8673,11 +8673,11 @@
       <c r="I126">
         <v>72</v>
       </c>
-      <c r="J126" s="12">
+      <c r="J126" s="11">
         <f t="shared" si="32"/>
         <v>-1</v>
       </c>
-      <c r="K126" s="25"/>
+      <c r="K126" s="24"/>
       <c r="L126" t="str">
         <f t="shared" si="21"/>
         <v/>
@@ -8717,7 +8717,7 @@
       <c r="B127" s="2" t="s">
         <v>89</v>
       </c>
-      <c r="C127" s="23">
+      <c r="C127" s="22">
         <v>34</v>
       </c>
       <c r="D127" s="2">
@@ -8729,7 +8729,7 @@
       <c r="F127" s="2">
         <v>16</v>
       </c>
-      <c r="G127" s="23">
+      <c r="G127" s="22">
         <f t="shared" si="36"/>
         <v>48</v>
       </c>
@@ -8739,11 +8739,11 @@
       <c r="I127" s="2">
         <v>56</v>
       </c>
-      <c r="J127" s="23">
+      <c r="J127" s="22">
         <f t="shared" si="32"/>
         <v>-5</v>
       </c>
-      <c r="K127" s="25"/>
+      <c r="K127" s="24"/>
       <c r="L127" t="str">
         <f t="shared" si="21"/>
         <v/>
@@ -8783,7 +8783,7 @@
       <c r="B128" t="s">
         <v>90</v>
       </c>
-      <c r="C128" s="12">
+      <c r="C128" s="11">
         <v>34</v>
       </c>
       <c r="D128">
@@ -8795,7 +8795,7 @@
       <c r="F128">
         <v>13</v>
       </c>
-      <c r="G128" s="12">
+      <c r="G128" s="11">
         <f t="shared" si="36"/>
         <v>45</v>
       </c>
@@ -8805,11 +8805,11 @@
       <c r="I128">
         <v>41</v>
       </c>
-      <c r="J128" s="12">
+      <c r="J128" s="11">
         <f t="shared" si="32"/>
         <v>-3</v>
       </c>
-      <c r="K128" s="25"/>
+      <c r="K128" s="24"/>
       <c r="L128" t="str">
         <f t="shared" si="21"/>
         <v/>
@@ -8849,7 +8849,7 @@
       <c r="B129" t="s">
         <v>91</v>
       </c>
-      <c r="C129" s="12">
+      <c r="C129" s="11">
         <v>34</v>
       </c>
       <c r="D129">
@@ -8861,7 +8861,7 @@
       <c r="F129">
         <v>18</v>
       </c>
-      <c r="G129" s="12">
+      <c r="G129" s="11">
         <f t="shared" si="36"/>
         <v>42</v>
       </c>
@@ -8871,11 +8871,11 @@
       <c r="I129">
         <v>76</v>
       </c>
-      <c r="J129" s="12">
+      <c r="J129" s="11">
         <f t="shared" si="32"/>
         <v>-14</v>
       </c>
-      <c r="K129" s="25"/>
+      <c r="K129" s="24"/>
       <c r="L129" t="str">
         <f t="shared" si="21"/>
         <v/>
@@ -8915,7 +8915,7 @@
       <c r="B130" t="s">
         <v>8</v>
       </c>
-      <c r="C130" s="12">
+      <c r="C130" s="11">
         <v>34</v>
       </c>
       <c r="D130">
@@ -8927,7 +8927,7 @@
       <c r="F130">
         <v>16</v>
       </c>
-      <c r="G130" s="12">
+      <c r="G130" s="11">
         <f t="shared" si="36"/>
         <v>38</v>
       </c>
@@ -8937,11 +8937,11 @@
       <c r="I130">
         <v>56</v>
       </c>
-      <c r="J130" s="12">
+      <c r="J130" s="11">
         <f t="shared" si="32"/>
         <v>-4</v>
       </c>
-      <c r="K130" s="25"/>
+      <c r="K130" s="24"/>
       <c r="L130" t="str">
         <f t="shared" si="21"/>
         <v/>
@@ -8981,7 +8981,7 @@
       <c r="B131" t="s">
         <v>92</v>
       </c>
-      <c r="C131" s="12">
+      <c r="C131" s="11">
         <v>34</v>
       </c>
       <c r="D131">
@@ -8993,7 +8993,7 @@
       <c r="F131">
         <v>16</v>
       </c>
-      <c r="G131" s="12">
+      <c r="G131" s="11">
         <f t="shared" si="36"/>
         <v>36</v>
       </c>
@@ -9003,11 +9003,11 @@
       <c r="I131">
         <v>72</v>
       </c>
-      <c r="J131" s="12">
+      <c r="J131" s="11">
         <f t="shared" si="32"/>
         <v>-20</v>
       </c>
-      <c r="K131" s="25"/>
+      <c r="K131" s="24"/>
       <c r="L131" t="str">
         <f t="shared" si="21"/>
         <v/>
@@ -9047,7 +9047,7 @@
       <c r="B132" s="3" t="s">
         <v>93</v>
       </c>
-      <c r="C132" s="13">
+      <c r="C132" s="12">
         <v>34</v>
       </c>
       <c r="D132" s="3">
@@ -9059,7 +9059,7 @@
       <c r="F132" s="3">
         <v>19</v>
       </c>
-      <c r="G132" s="13">
+      <c r="G132" s="12">
         <f t="shared" si="36"/>
         <v>35</v>
       </c>
@@ -9069,11 +9069,11 @@
       <c r="I132" s="3">
         <v>71</v>
       </c>
-      <c r="J132" s="13">
+      <c r="J132" s="12">
         <f t="shared" si="32"/>
         <v>-22</v>
       </c>
-      <c r="K132" s="25"/>
+      <c r="K132" s="24"/>
       <c r="L132" t="str">
         <f t="shared" si="21"/>
         <v/>
@@ -9113,7 +9113,7 @@
       <c r="B133" s="3" t="s">
         <v>94</v>
       </c>
-      <c r="C133" s="13">
+      <c r="C133" s="12">
         <v>34</v>
       </c>
       <c r="D133" s="3">
@@ -9125,7 +9125,7 @@
       <c r="F133" s="3">
         <v>17</v>
       </c>
-      <c r="G133" s="13">
+      <c r="G133" s="12">
         <f t="shared" si="36"/>
         <v>33</v>
       </c>
@@ -9135,11 +9135,11 @@
       <c r="I133" s="3">
         <v>58</v>
       </c>
-      <c r="J133" s="13">
+      <c r="J133" s="12">
         <f t="shared" si="32"/>
         <v>-11</v>
       </c>
-      <c r="K133" s="25"/>
+      <c r="K133" s="24"/>
       <c r="L133" t="str">
         <f t="shared" ref="L133:L196" si="37">IF(A133="","",A133)</f>
         <v/>
@@ -9179,7 +9179,7 @@
       <c r="B134" s="4" t="s">
         <v>69</v>
       </c>
-      <c r="C134" s="14">
+      <c r="C134" s="13">
         <v>34</v>
       </c>
       <c r="D134" s="4">
@@ -9191,7 +9191,7 @@
       <c r="F134" s="4">
         <v>17</v>
       </c>
-      <c r="G134" s="14">
+      <c r="G134" s="13">
         <f t="shared" si="36"/>
         <v>33</v>
       </c>
@@ -9201,11 +9201,11 @@
       <c r="I134" s="4">
         <v>65</v>
       </c>
-      <c r="J134" s="14">
+      <c r="J134" s="13">
         <f t="shared" si="32"/>
         <v>-15</v>
       </c>
-      <c r="K134" s="25"/>
+      <c r="K134" s="24"/>
       <c r="L134" t="str">
         <f t="shared" si="37"/>
         <v/>
@@ -9245,7 +9245,7 @@
       <c r="B135" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="C135" s="14">
+      <c r="C135" s="13">
         <v>34</v>
       </c>
       <c r="D135" s="4">
@@ -9257,7 +9257,7 @@
       <c r="F135" s="4">
         <v>21</v>
       </c>
-      <c r="G135" s="14">
+      <c r="G135" s="13">
         <f t="shared" si="36"/>
         <v>27</v>
       </c>
@@ -9267,11 +9267,11 @@
       <c r="I135" s="4">
         <v>61</v>
       </c>
-      <c r="J135" s="14">
+      <c r="J135" s="13">
         <f t="shared" si="32"/>
         <v>-36</v>
       </c>
-      <c r="K135" s="25"/>
+      <c r="K135" s="24"/>
       <c r="L135" t="str">
         <f t="shared" si="37"/>
         <v/>
@@ -9320,7 +9320,7 @@
       <c r="B137" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="C137" s="9">
+      <c r="C137" s="8">
         <v>34</v>
       </c>
       <c r="D137" s="1">
@@ -9333,7 +9333,7 @@
         <f>C137-D137-E137</f>
         <v>10</v>
       </c>
-      <c r="G137" s="9">
+      <c r="G137" s="8">
         <f>D137*3+E137</f>
         <v>66</v>
       </c>
@@ -9343,11 +9343,11 @@
       <c r="I137" s="1">
         <v>53</v>
       </c>
-      <c r="J137" s="9">
+      <c r="J137" s="8">
         <f>H137-I137</f>
         <v>39</v>
       </c>
-      <c r="K137" s="25"/>
+      <c r="K137" s="24"/>
       <c r="L137" t="str">
         <f t="shared" si="37"/>
         <v>2023/24</v>
@@ -9368,7 +9368,7 @@
         <f>N137-O137-P137</f>
         <v>7</v>
       </c>
-      <c r="R137" s="9">
+      <c r="R137" s="8">
         <f t="shared" ref="R137:R154" si="38">O137*3+P137*1</f>
         <v>71</v>
       </c>
@@ -9384,37 +9384,37 @@
       </c>
     </row>
     <row r="138" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="B138" s="8" t="s">
+      <c r="B138" s="7" t="s">
         <v>98</v>
       </c>
-      <c r="C138" s="22">
-        <v>34</v>
-      </c>
-      <c r="D138" s="8">
+      <c r="C138" s="21">
+        <v>34</v>
+      </c>
+      <c r="D138" s="7">
         <v>19</v>
       </c>
-      <c r="E138" s="8">
+      <c r="E138" s="7">
         <v>6</v>
       </c>
-      <c r="F138" s="8">
+      <c r="F138" s="7">
         <f t="shared" ref="F138:F154" si="39">C138-D138-E138</f>
         <v>9</v>
       </c>
-      <c r="G138" s="22">
+      <c r="G138" s="21">
         <f t="shared" ref="G138:G154" si="40">D138*3+E138</f>
         <v>63</v>
       </c>
-      <c r="H138" s="8">
+      <c r="H138" s="7">
         <v>72</v>
       </c>
-      <c r="I138" s="8">
+      <c r="I138" s="7">
         <v>43</v>
       </c>
-      <c r="J138" s="22">
+      <c r="J138" s="21">
         <f t="shared" ref="J138:J154" si="41">H138-I138</f>
         <v>29</v>
       </c>
-      <c r="K138" s="25"/>
+      <c r="K138" s="24"/>
       <c r="L138" t="str">
         <f t="shared" si="37"/>
         <v/>
@@ -9435,7 +9435,7 @@
         <f t="shared" ref="Q138:Q154" si="42">N138-O138-P138</f>
         <v>5</v>
       </c>
-      <c r="R138" s="23">
+      <c r="R138" s="22">
         <f t="shared" si="38"/>
         <v>69</v>
       </c>
@@ -9501,7 +9501,7 @@
         <f t="shared" si="42"/>
         <v>7</v>
       </c>
-      <c r="R139" s="23">
+      <c r="R139" s="22">
         <f t="shared" si="38"/>
         <v>67</v>
       </c>
@@ -9586,7 +9586,7 @@
       <c r="B141" t="s">
         <v>88</v>
       </c>
-      <c r="C141" s="12">
+      <c r="C141" s="11">
         <v>34</v>
       </c>
       <c r="D141">
@@ -9599,7 +9599,7 @@
         <f t="shared" si="39"/>
         <v>14</v>
       </c>
-      <c r="G141" s="12">
+      <c r="G141" s="11">
         <f t="shared" si="40"/>
         <v>56</v>
       </c>
@@ -9609,11 +9609,11 @@
       <c r="I141">
         <v>66</v>
       </c>
-      <c r="J141" s="12">
+      <c r="J141" s="11">
         <f t="shared" si="41"/>
         <v>15</v>
       </c>
-      <c r="K141" s="25"/>
+      <c r="K141" s="24"/>
       <c r="L141" t="str">
         <f t="shared" si="37"/>
         <v/>
@@ -9634,7 +9634,7 @@
         <f t="shared" si="42"/>
         <v>9</v>
       </c>
-      <c r="R141" s="12">
+      <c r="R141" s="11">
         <f t="shared" si="38"/>
         <v>61</v>
       </c>
@@ -9700,7 +9700,7 @@
         <f t="shared" si="42"/>
         <v>10</v>
       </c>
-      <c r="R142" s="12">
+      <c r="R142" s="11">
         <f>O142*3+P142*1</f>
         <v>58</v>
       </c>
@@ -9719,7 +9719,7 @@
       <c r="B143" t="s">
         <v>89</v>
       </c>
-      <c r="C143" s="12">
+      <c r="C143" s="11">
         <v>34</v>
       </c>
       <c r="D143">
@@ -9732,7 +9732,7 @@
         <f t="shared" si="39"/>
         <v>10</v>
       </c>
-      <c r="G143" s="12">
+      <c r="G143" s="11">
         <f t="shared" si="40"/>
         <v>52</v>
       </c>
@@ -9742,11 +9742,11 @@
       <c r="I143">
         <v>45</v>
       </c>
-      <c r="J143" s="12">
+      <c r="J143" s="11">
         <f t="shared" si="41"/>
         <v>17</v>
       </c>
-      <c r="K143" s="25"/>
+      <c r="K143" s="24"/>
       <c r="L143" t="str">
         <f t="shared" si="37"/>
         <v/>
@@ -9767,7 +9767,7 @@
         <f t="shared" si="42"/>
         <v>10</v>
       </c>
-      <c r="R143" s="12">
+      <c r="R143" s="11">
         <f t="shared" si="38"/>
         <v>56</v>
       </c>
@@ -9786,7 +9786,7 @@
       <c r="B144" t="s">
         <v>27</v>
       </c>
-      <c r="C144" s="12">
+      <c r="C144" s="11">
         <v>34</v>
       </c>
       <c r="D144">
@@ -9799,7 +9799,7 @@
         <f t="shared" si="39"/>
         <v>10</v>
       </c>
-      <c r="G144" s="12">
+      <c r="G144" s="11">
         <f t="shared" si="40"/>
         <v>52</v>
       </c>
@@ -9809,11 +9809,11 @@
       <c r="I144">
         <v>53</v>
       </c>
-      <c r="J144" s="12">
+      <c r="J144" s="11">
         <f t="shared" si="41"/>
         <v>7</v>
       </c>
-      <c r="K144" s="25"/>
+      <c r="K144" s="24"/>
       <c r="L144" t="str">
         <f t="shared" si="37"/>
         <v/>
@@ -9834,7 +9834,7 @@
         <f t="shared" si="42"/>
         <v>16</v>
       </c>
-      <c r="R144" s="12">
+      <c r="R144" s="11">
         <f t="shared" si="38"/>
         <v>50</v>
       </c>
@@ -9853,7 +9853,7 @@
       <c r="B145" t="s">
         <v>87</v>
       </c>
-      <c r="C145" s="12">
+      <c r="C145" s="11">
         <v>34</v>
       </c>
       <c r="D145">
@@ -9866,7 +9866,7 @@
         <f t="shared" si="39"/>
         <v>14</v>
       </c>
-      <c r="G145" s="12">
+      <c r="G145" s="11">
         <f t="shared" si="40"/>
         <v>48</v>
       </c>
@@ -9876,11 +9876,11 @@
       <c r="I145">
         <v>42</v>
       </c>
-      <c r="J145" s="12">
+      <c r="J145" s="11">
         <f t="shared" si="41"/>
         <v>19</v>
       </c>
-      <c r="K145" s="25"/>
+      <c r="K145" s="24"/>
       <c r="L145" t="str">
         <f t="shared" si="37"/>
         <v/>
@@ -9901,7 +9901,7 @@
         <f t="shared" si="42"/>
         <v>13</v>
       </c>
-      <c r="R145" s="12">
+      <c r="R145" s="11">
         <f t="shared" si="38"/>
         <v>47</v>
       </c>
@@ -9917,37 +9917,37 @@
       </c>
     </row>
     <row r="146" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="B146" s="20" t="s">
+      <c r="B146" s="19" t="s">
         <v>85</v>
       </c>
-      <c r="C146" s="21">
-        <v>34</v>
-      </c>
-      <c r="D146" s="20">
+      <c r="C146" s="20">
+        <v>34</v>
+      </c>
+      <c r="D146" s="19">
         <v>14</v>
       </c>
-      <c r="E146" s="20">
+      <c r="E146" s="19">
         <v>6</v>
       </c>
-      <c r="F146" s="20">
+      <c r="F146" s="19">
         <f t="shared" si="39"/>
         <v>14</v>
       </c>
-      <c r="G146" s="21">
+      <c r="G146" s="20">
         <f t="shared" si="40"/>
         <v>48</v>
       </c>
-      <c r="H146" s="20">
+      <c r="H146" s="19">
         <v>60</v>
       </c>
-      <c r="I146" s="20">
+      <c r="I146" s="19">
         <v>62</v>
       </c>
-      <c r="J146" s="21">
+      <c r="J146" s="20">
         <f t="shared" si="41"/>
         <v>-2</v>
       </c>
-      <c r="K146" s="25"/>
+      <c r="K146" s="24"/>
       <c r="L146" t="str">
         <f t="shared" si="37"/>
         <v/>
@@ -9968,7 +9968,7 @@
         <f t="shared" si="42"/>
         <v>13</v>
       </c>
-      <c r="R146" s="12">
+      <c r="R146" s="11">
         <f t="shared" si="38"/>
         <v>47</v>
       </c>
@@ -9987,7 +9987,7 @@
       <c r="B147" t="s">
         <v>100</v>
       </c>
-      <c r="C147" s="12">
+      <c r="C147" s="11">
         <v>34</v>
       </c>
       <c r="D147">
@@ -10000,7 +10000,7 @@
         <f t="shared" si="39"/>
         <v>12</v>
       </c>
-      <c r="G147" s="12">
+      <c r="G147" s="11">
         <f t="shared" si="40"/>
         <v>48</v>
       </c>
@@ -10010,11 +10010,11 @@
       <c r="I147">
         <v>62</v>
       </c>
-      <c r="J147" s="12">
+      <c r="J147" s="11">
         <f t="shared" si="41"/>
         <v>-5</v>
       </c>
-      <c r="K147" s="25"/>
+      <c r="K147" s="24"/>
       <c r="L147" t="str">
         <f t="shared" si="37"/>
         <v/>
@@ -10035,7 +10035,7 @@
         <f t="shared" si="42"/>
         <v>17</v>
       </c>
-      <c r="R147" s="12">
+      <c r="R147" s="11">
         <f t="shared" si="38"/>
         <v>47</v>
       </c>
@@ -10054,7 +10054,7 @@
       <c r="B148" t="s">
         <v>68</v>
       </c>
-      <c r="C148" s="12">
+      <c r="C148" s="11">
         <v>34</v>
       </c>
       <c r="D148">
@@ -10067,7 +10067,7 @@
         <f t="shared" si="39"/>
         <v>15</v>
       </c>
-      <c r="G148" s="12">
+      <c r="G148" s="11">
         <f t="shared" si="40"/>
         <v>47</v>
       </c>
@@ -10077,11 +10077,11 @@
       <c r="I148">
         <v>67</v>
       </c>
-      <c r="J148" s="12">
+      <c r="J148" s="11">
         <f t="shared" si="41"/>
         <v>-5</v>
       </c>
-      <c r="K148" s="25"/>
+      <c r="K148" s="24"/>
       <c r="L148" t="str">
         <f t="shared" si="37"/>
         <v/>
@@ -10102,7 +10102,7 @@
         <f t="shared" si="42"/>
         <v>13</v>
       </c>
-      <c r="R148" s="12">
+      <c r="R148" s="11">
         <f>O148*3+P148*1</f>
         <v>47</v>
       </c>
@@ -10121,7 +10121,7 @@
       <c r="B149" t="s">
         <v>101</v>
       </c>
-      <c r="C149" s="12">
+      <c r="C149" s="11">
         <v>34</v>
       </c>
       <c r="D149">
@@ -10134,7 +10134,7 @@
         <f t="shared" si="39"/>
         <v>15</v>
       </c>
-      <c r="G149" s="12">
+      <c r="G149" s="11">
         <f t="shared" si="40"/>
         <v>47</v>
       </c>
@@ -10144,11 +10144,11 @@
       <c r="I149">
         <v>54</v>
       </c>
-      <c r="J149" s="12">
+      <c r="J149" s="11">
         <f t="shared" si="41"/>
         <v>-5</v>
       </c>
-      <c r="K149" s="25"/>
+      <c r="K149" s="24"/>
       <c r="L149" t="str">
         <f t="shared" si="37"/>
         <v/>
@@ -10169,7 +10169,7 @@
         <f t="shared" si="42"/>
         <v>14</v>
       </c>
-      <c r="R149" s="12">
+      <c r="R149" s="11">
         <f t="shared" si="38"/>
         <v>36</v>
       </c>
@@ -10188,7 +10188,7 @@
       <c r="B150" t="s">
         <v>102</v>
       </c>
-      <c r="C150" s="12">
+      <c r="C150" s="11">
         <v>34</v>
       </c>
       <c r="D150">
@@ -10201,7 +10201,7 @@
         <f t="shared" si="39"/>
         <v>13</v>
       </c>
-      <c r="G150" s="12">
+      <c r="G150" s="11">
         <f t="shared" si="40"/>
         <v>45</v>
       </c>
@@ -10211,11 +10211,11 @@
       <c r="I150">
         <v>73</v>
       </c>
-      <c r="J150" s="12">
+      <c r="J150" s="11">
         <f t="shared" si="41"/>
         <v>-17</v>
       </c>
-      <c r="K150" s="25"/>
+      <c r="K150" s="24"/>
       <c r="L150" t="str">
         <f t="shared" si="37"/>
         <v/>
@@ -10236,7 +10236,7 @@
         <f t="shared" si="42"/>
         <v>18</v>
       </c>
-      <c r="R150" s="12">
+      <c r="R150" s="11">
         <f>O150*3+P150*1</f>
         <v>36</v>
       </c>
@@ -10255,7 +10255,7 @@
       <c r="B151" s="3" t="s">
         <v>90</v>
       </c>
-      <c r="C151" s="13">
+      <c r="C151" s="12">
         <v>34</v>
       </c>
       <c r="D151" s="3">
@@ -10268,7 +10268,7 @@
         <f t="shared" si="39"/>
         <v>16</v>
       </c>
-      <c r="G151" s="13">
+      <c r="G151" s="12">
         <f t="shared" si="40"/>
         <v>44</v>
       </c>
@@ -10278,11 +10278,11 @@
       <c r="I151" s="3">
         <v>64</v>
       </c>
-      <c r="J151" s="13">
+      <c r="J151" s="12">
         <f t="shared" si="41"/>
         <v>-8</v>
       </c>
-      <c r="K151" s="25"/>
+      <c r="K151" s="24"/>
       <c r="L151" t="str">
         <f t="shared" si="37"/>
         <v/>
@@ -10303,7 +10303,7 @@
         <f t="shared" si="42"/>
         <v>19</v>
       </c>
-      <c r="R151" s="13">
+      <c r="R151" s="12">
         <f>O151*3+P151*1-1</f>
         <v>30</v>
       </c>
@@ -10322,7 +10322,7 @@
       <c r="B152" s="3" t="s">
         <v>103</v>
       </c>
-      <c r="C152" s="13">
+      <c r="C152" s="12">
         <v>34</v>
       </c>
       <c r="D152" s="3">
@@ -10335,7 +10335,7 @@
         <f t="shared" si="39"/>
         <v>21</v>
       </c>
-      <c r="G152" s="13">
+      <c r="G152" s="12">
         <f t="shared" si="40"/>
         <v>33</v>
       </c>
@@ -10345,11 +10345,11 @@
       <c r="I152" s="3">
         <v>87</v>
       </c>
-      <c r="J152" s="13">
+      <c r="J152" s="12">
         <f t="shared" si="41"/>
         <v>-42</v>
       </c>
-      <c r="K152" s="25"/>
+      <c r="K152" s="24"/>
       <c r="L152" t="str">
         <f t="shared" si="37"/>
         <v/>
@@ -10370,7 +10370,7 @@
         <f t="shared" si="42"/>
         <v>21</v>
       </c>
-      <c r="R152" s="13">
+      <c r="R152" s="12">
         <f t="shared" si="38"/>
         <v>29</v>
       </c>
@@ -10389,7 +10389,7 @@
       <c r="B153" s="4" t="s">
         <v>104</v>
       </c>
-      <c r="C153" s="14">
+      <c r="C153" s="13">
         <v>34</v>
       </c>
       <c r="D153" s="4">
@@ -10402,7 +10402,7 @@
         <f t="shared" si="39"/>
         <v>21</v>
       </c>
-      <c r="G153" s="14">
+      <c r="G153" s="13">
         <f t="shared" si="40"/>
         <v>25</v>
       </c>
@@ -10412,11 +10412,11 @@
       <c r="I153" s="4">
         <v>70</v>
       </c>
-      <c r="J153" s="14">
+      <c r="J153" s="13">
         <f t="shared" si="41"/>
         <v>-26</v>
       </c>
-      <c r="K153" s="25"/>
+      <c r="K153" s="24"/>
       <c r="L153" t="str">
         <f t="shared" si="37"/>
         <v/>
@@ -10437,7 +10437,7 @@
         <f t="shared" si="42"/>
         <v>22</v>
       </c>
-      <c r="R153" s="14">
+      <c r="R153" s="13">
         <f t="shared" si="38"/>
         <v>26</v>
       </c>
@@ -10456,7 +10456,7 @@
       <c r="B154" s="4" t="s">
         <v>105</v>
       </c>
-      <c r="C154" s="14">
+      <c r="C154" s="13">
         <v>34</v>
       </c>
       <c r="D154" s="4">
@@ -10469,7 +10469,7 @@
         <f t="shared" si="39"/>
         <v>26</v>
       </c>
-      <c r="G154" s="14">
+      <c r="G154" s="13">
         <f t="shared" si="40"/>
         <v>14</v>
       </c>
@@ -10479,11 +10479,11 @@
       <c r="I154" s="4">
         <v>108</v>
       </c>
-      <c r="J154" s="14">
+      <c r="J154" s="13">
         <f t="shared" si="41"/>
         <v>-79</v>
       </c>
-      <c r="K154" s="25"/>
+      <c r="K154" s="24"/>
       <c r="L154" t="str">
         <f t="shared" si="37"/>
         <v/>
@@ -10504,7 +10504,7 @@
         <f t="shared" si="42"/>
         <v>26</v>
       </c>
-      <c r="R154" s="14">
+      <c r="R154" s="13">
         <f t="shared" si="38"/>
         <v>20</v>
       </c>
@@ -11613,15 +11613,15 @@
         <f t="shared" si="37"/>
         <v/>
       </c>
-      <c r="M174" s="12"/>
-      <c r="N174" s="12"/>
-      <c r="O174" s="12"/>
-      <c r="P174" s="12"/>
-      <c r="Q174" s="12"/>
-      <c r="R174" s="12"/>
-      <c r="S174" s="12"/>
-      <c r="T174" s="12"/>
-      <c r="U174" s="12"/>
+      <c r="M174" s="11"/>
+      <c r="N174" s="11"/>
+      <c r="O174" s="11"/>
+      <c r="P174" s="11"/>
+      <c r="Q174" s="11"/>
+      <c r="R174" s="11"/>
+      <c r="S174" s="11"/>
+      <c r="T174" s="11"/>
+      <c r="U174" s="11"/>
     </row>
     <row r="175" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A175" t="s">
@@ -11643,7 +11643,7 @@
         <f>34-D175-E175</f>
         <v>7</v>
       </c>
-      <c r="G175" s="12">
+      <c r="G175" s="11">
         <f>D175*3+E175</f>
         <v>67</v>
       </c>
@@ -11677,7 +11677,7 @@
         <f>34-O175-P175</f>
         <v>5</v>
       </c>
-      <c r="R175" s="12">
+      <c r="R175" s="11">
         <f>O175*3+P175</f>
         <v>73</v>
       </c>
@@ -11709,7 +11709,7 @@
         <f t="shared" ref="F176:F192" si="44">34-D176-E176</f>
         <v>6</v>
       </c>
-      <c r="G176" s="12">
+      <c r="G176" s="11">
         <f t="shared" ref="G176:G192" si="45">D176*3+E176</f>
         <v>62</v>
       </c>
@@ -11743,7 +11743,7 @@
         <f t="shared" ref="Q176:Q192" si="47">34-O176-P176</f>
         <v>6</v>
       </c>
-      <c r="R176" s="12">
+      <c r="R176" s="11">
         <f t="shared" ref="R176:R192" si="48">O176*3+P176</f>
         <v>68</v>
       </c>
@@ -11775,7 +11775,7 @@
         <f t="shared" si="44"/>
         <v>11</v>
       </c>
-      <c r="G177" s="12">
+      <c r="G177" s="11">
         <f t="shared" si="45"/>
         <v>61</v>
       </c>
@@ -11809,7 +11809,7 @@
         <f t="shared" si="47"/>
         <v>8</v>
       </c>
-      <c r="R177" s="12">
+      <c r="R177" s="11">
         <f t="shared" si="48"/>
         <v>68</v>
       </c>
@@ -11841,7 +11841,7 @@
         <f t="shared" si="44"/>
         <v>8</v>
       </c>
-      <c r="G178" s="12">
+      <c r="G178" s="11">
         <f t="shared" si="45"/>
         <v>60</v>
       </c>
@@ -11875,7 +11875,7 @@
         <f t="shared" si="47"/>
         <v>8</v>
       </c>
-      <c r="R178" s="12">
+      <c r="R178" s="11">
         <f t="shared" si="48"/>
         <v>64</v>
       </c>
@@ -11907,7 +11907,7 @@
         <f t="shared" si="44"/>
         <v>12</v>
       </c>
-      <c r="G179" s="12">
+      <c r="G179" s="11">
         <f t="shared" si="45"/>
         <v>56</v>
       </c>
@@ -11941,7 +11941,7 @@
         <f t="shared" si="47"/>
         <v>7</v>
       </c>
-      <c r="R179" s="12">
+      <c r="R179" s="11">
         <f t="shared" si="48"/>
         <v>61</v>
       </c>
@@ -11973,7 +11973,7 @@
         <f t="shared" si="44"/>
         <v>14</v>
       </c>
-      <c r="G180" s="12">
+      <c r="G180" s="11">
         <f t="shared" si="45"/>
         <v>54</v>
       </c>
@@ -12007,7 +12007,7 @@
         <f t="shared" si="47"/>
         <v>10</v>
       </c>
-      <c r="R180" s="12">
+      <c r="R180" s="11">
         <f t="shared" si="48"/>
         <v>54</v>
       </c>
@@ -12039,7 +12039,7 @@
         <f t="shared" si="44"/>
         <v>10</v>
       </c>
-      <c r="G181" s="12">
+      <c r="G181" s="11">
         <f t="shared" si="45"/>
         <v>52</v>
       </c>
@@ -12073,7 +12073,7 @@
         <f t="shared" si="47"/>
         <v>11</v>
       </c>
-      <c r="R181" s="12">
+      <c r="R181" s="11">
         <f t="shared" si="48"/>
         <v>53</v>
       </c>
@@ -12105,7 +12105,7 @@
         <f t="shared" si="44"/>
         <v>12</v>
       </c>
-      <c r="G182" s="12">
+      <c r="G182" s="11">
         <f t="shared" si="45"/>
         <v>52</v>
       </c>
@@ -12139,7 +12139,7 @@
         <f t="shared" si="47"/>
         <v>13</v>
       </c>
-      <c r="R182" s="12">
+      <c r="R182" s="11">
         <f t="shared" si="48"/>
         <v>51</v>
       </c>
@@ -12171,7 +12171,7 @@
         <f t="shared" si="44"/>
         <v>12</v>
       </c>
-      <c r="G183" s="12">
+      <c r="G183" s="11">
         <f t="shared" si="45"/>
         <v>50</v>
       </c>
@@ -12205,7 +12205,7 @@
         <f t="shared" si="47"/>
         <v>14</v>
       </c>
-      <c r="R183" s="12">
+      <c r="R183" s="11">
         <f t="shared" si="48"/>
         <v>48</v>
       </c>
@@ -12237,7 +12237,7 @@
         <f t="shared" si="44"/>
         <v>13</v>
       </c>
-      <c r="G184" s="12">
+      <c r="G184" s="11">
         <f t="shared" si="45"/>
         <v>49</v>
       </c>
@@ -12271,7 +12271,7 @@
         <f t="shared" si="47"/>
         <v>14</v>
       </c>
-      <c r="R184" s="12">
+      <c r="R184" s="11">
         <f t="shared" si="48"/>
         <v>44</v>
       </c>
@@ -12303,7 +12303,7 @@
         <f t="shared" si="44"/>
         <v>14</v>
       </c>
-      <c r="G185" s="12">
+      <c r="G185" s="11">
         <f t="shared" si="45"/>
         <v>48</v>
       </c>
@@ -12337,7 +12337,7 @@
         <f t="shared" si="47"/>
         <v>17</v>
       </c>
-      <c r="R185" s="12">
+      <c r="R185" s="11">
         <f t="shared" si="48"/>
         <v>39</v>
       </c>
@@ -12369,7 +12369,7 @@
         <f t="shared" si="44"/>
         <v>15</v>
       </c>
-      <c r="G186" s="12">
+      <c r="G186" s="11">
         <f t="shared" si="45"/>
         <v>47</v>
       </c>
@@ -12403,7 +12403,7 @@
         <f t="shared" si="47"/>
         <v>16</v>
       </c>
-      <c r="R186" s="12">
+      <c r="R186" s="11">
         <f t="shared" si="48"/>
         <v>38</v>
       </c>
@@ -12435,7 +12435,7 @@
         <f t="shared" si="44"/>
         <v>16</v>
       </c>
-      <c r="G187" s="12">
+      <c r="G187" s="11">
         <f t="shared" si="45"/>
         <v>44</v>
       </c>
@@ -12469,7 +12469,7 @@
         <f t="shared" si="47"/>
         <v>17</v>
       </c>
-      <c r="R187" s="12">
+      <c r="R187" s="11">
         <f t="shared" si="48"/>
         <v>37</v>
       </c>
@@ -12501,7 +12501,7 @@
         <f t="shared" si="44"/>
         <v>18</v>
       </c>
-      <c r="G188" s="12">
+      <c r="G188" s="11">
         <f t="shared" si="45"/>
         <v>40</v>
       </c>
@@ -12535,7 +12535,7 @@
         <f t="shared" si="47"/>
         <v>18</v>
       </c>
-      <c r="R188" s="12">
+      <c r="R188" s="11">
         <f t="shared" si="48"/>
         <v>36</v>
       </c>
@@ -12567,7 +12567,7 @@
         <f t="shared" si="44"/>
         <v>16</v>
       </c>
-      <c r="G189" s="12">
+      <c r="G189" s="11">
         <f t="shared" si="45"/>
         <v>40</v>
       </c>
@@ -12601,7 +12601,7 @@
         <f t="shared" si="47"/>
         <v>20</v>
       </c>
-      <c r="R189" s="12">
+      <c r="R189" s="11">
         <f t="shared" si="48"/>
         <v>34</v>
       </c>
@@ -12633,7 +12633,7 @@
         <f t="shared" si="44"/>
         <v>18</v>
       </c>
-      <c r="G190" s="12">
+      <c r="G190" s="11">
         <f t="shared" si="45"/>
         <v>40</v>
       </c>
@@ -12667,7 +12667,7 @@
         <f t="shared" si="47"/>
         <v>20</v>
       </c>
-      <c r="R190" s="12">
+      <c r="R190" s="11">
         <f t="shared" si="48"/>
         <v>32</v>
       </c>
@@ -12699,7 +12699,7 @@
         <f t="shared" si="44"/>
         <v>19</v>
       </c>
-      <c r="G191" s="12">
+      <c r="G191" s="11">
         <f t="shared" si="45"/>
         <v>33</v>
       </c>
@@ -12733,7 +12733,7 @@
         <f t="shared" si="47"/>
         <v>19</v>
       </c>
-      <c r="R191" s="12">
+      <c r="R191" s="11">
         <f t="shared" si="48"/>
         <v>31</v>
       </c>
@@ -12765,7 +12765,7 @@
         <f t="shared" si="44"/>
         <v>29</v>
       </c>
-      <c r="G192" s="12">
+      <c r="G192" s="11">
         <f t="shared" si="45"/>
         <v>7</v>
       </c>
@@ -12799,7 +12799,7 @@
         <f t="shared" si="47"/>
         <v>21</v>
       </c>
-      <c r="R192" s="12">
+      <c r="R192" s="11">
         <f t="shared" si="48"/>
         <v>25</v>
       </c>
@@ -12815,7 +12815,7 @@
       </c>
     </row>
     <row r="193" spans="7:12" x14ac:dyDescent="0.3">
-      <c r="G193" s="12"/>
+      <c r="G193" s="11"/>
       <c r="L193" t="str">
         <f t="shared" si="37"/>
         <v/>

</xml_diff>